<commit_message>
upgrade the styles export on border
</commit_message>
<xml_diff>
--- a/3-Dev/DevApp/Files/CellFormat.xlsx
+++ b/3-Dev/DevApp/Files/CellFormat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/3-Dev/DevApp/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F7D5EDD-9E68-4A31-B616-BC8AD40C60D1}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{201EE4BC-62F0-4671-9B43-9D1EBCE6EE65}"/>
   <bookViews>
-    <workbookView xWindow="9030" yWindow="4710" windowWidth="19065" windowHeight="9735" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
+    <workbookView xWindow="9375" yWindow="3915" windowWidth="18150" windowHeight="13170" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
   <si>
     <t>value</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>y</t>
+  </si>
+  <si>
+    <t>hello</t>
   </si>
 </sst>
 </file>
@@ -86,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -94,15 +97,66 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="1" diagonalDown="1">
+      <left style="thin">
+        <color rgb="FF0070C0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF0070C0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF0070C0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF0070C0"/>
+      </bottom>
+      <diagonal style="thin">
+        <color rgb="FF0070C0"/>
+      </diagonal>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,10 +495,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C34316-5981-45DA-B1A5-D1338D5ADA96}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -452,33 +506,43 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="1">
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>12.34</v>
+      </c>
+      <c r="B2" s="4">
         <v>12</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
       </c>
+      <c r="D2" s="6">
+        <v>46001</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
       <c r="B3" s="3">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="1">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="5">
         <v>12</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
+      <c r="D4" s="7"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
add currency on GetcellValue
</commit_message>
<xml_diff>
--- a/3-Dev/DevApp/Files/CellFormat.xlsx
+++ b/3-Dev/DevApp/Files/CellFormat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/3-Dev/DevApp/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{201EE4BC-62F0-4671-9B43-9D1EBCE6EE65}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08EE0A04-37B8-4CAF-8EB8-B13BEB6AE0B5}"/>
   <bookViews>
-    <workbookView xWindow="9375" yWindow="3915" windowWidth="18150" windowHeight="13170" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
+    <workbookView xWindow="5205" yWindow="3330" windowWidth="20040" windowHeight="11445" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
   <si>
     <t>value</t>
   </si>
@@ -48,6 +48,12 @@
   </si>
   <si>
     <t>hello</t>
+  </si>
+  <si>
+    <t>er</t>
+  </si>
+  <si>
+    <t>formula</t>
   </si>
 </sst>
 </file>
@@ -63,7 +69,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -88,6 +94,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -148,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -157,6 +169,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,10 +508,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C34316-5981-45DA-B1A5-D1338D5ADA96}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -506,7 +519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>12.34</v>
       </c>
@@ -520,7 +533,7 @@
         <v>46001</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -528,7 +541,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="5">
         <v>12</v>
       </c>
@@ -537,17 +550,29 @@
       </c>
       <c r="D4" s="7"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>34</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7">
+        <f>B2+B3</f>
+        <v>57</v>
+      </c>
+      <c r="E7" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>